<commit_message>
feat: add some minor function for the modelling
</commit_message>
<xml_diff>
--- a/result/predicted_and_measured_proteomics.xlsx
+++ b/result/predicted_and_measured_proteomics.xlsx
@@ -538,7 +538,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1.533143450546697e-05</v>
+        <v>1.53314345054673e-05</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -559,7 +559,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1.533143450546697e-05</v>
+        <v>1.53314345054673e-05</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -580,7 +580,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1.533143450546697e-05</v>
+        <v>1.53314345054673e-05</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -620,7 +620,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>7.448518394754971e-06</v>
+        <v>7.448518394754906e-06</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.0002713682700173554</v>
+        <v>0.0002713682700173536</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -723,7 +723,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>4.86346396611867e-06</v>
+        <v>4.863463966118776e-06</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -742,7 +742,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>4.86346396611867e-06</v>
+        <v>4.863463966118776e-06</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -763,7 +763,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>4.86346396611867e-06</v>
+        <v>4.863463966118776e-06</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -784,7 +784,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>4.86346396611867e-06</v>
+        <v>4.863463966118776e-06</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -803,7 +803,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>4.86346396611867e-06</v>
+        <v>4.863463966118776e-06</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -908,7 +908,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>3.319190088557132e-05</v>
+        <v>3.319190088557111e-05</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -929,7 +929,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1.466320290074298e-05</v>
+        <v>1.466320290074288e-05</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1072,7 +1072,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>6.301819192898289e-06</v>
+        <v>6.301819192898404e-06</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -1093,7 +1093,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2.048077302484792e-05</v>
+        <v>2.04807730248483e-05</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>2.048077302484792e-05</v>
+        <v>2.04807730248483e-05</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -1131,7 +1131,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1.080536555789824e-06</v>
+        <v>1.0805365557899e-06</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -1194,7 +1194,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>3.381900951768773e-05</v>
+        <v>3.381900951768752e-05</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -1236,7 +1236,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>1.247135338319999e-07</v>
+        <v>1.24713533832e-07</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>4.448437580910157e-07</v>
+        <v>4.448437580910126e-07</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -1362,7 +1362,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>2.216462571093599e-08</v>
+        <v>2.216462571093601e-08</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -1404,7 +1404,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>4.86346396611867e-06</v>
+        <v>4.863463966118776e-06</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -1425,7 +1425,7 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>9.727049354915876e-06</v>
+        <v>9.727049354916089e-06</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -1446,7 +1446,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>2.034349670866593e-07</v>
+        <v>2.034349670866569e-07</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -1488,7 +1488,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>1.508489987805062e-06</v>
+        <v>1.508489987805044e-06</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -1778,7 +1778,7 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>2.048077302484792e-05</v>
+        <v>2.04807730248483e-05</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -1799,7 +1799,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>6.446627856529884e-06</v>
+        <v>6.446627856529883e-06</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -1881,7 +1881,7 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>4.723451690843427e-05</v>
+        <v>4.723451690843386e-05</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -2112,7 +2112,7 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>1.533143450546697e-05</v>
+        <v>1.53314345054673e-05</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -2217,7 +2217,7 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>3.232519274566961e-06</v>
+        <v>3.232519274566923e-06</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
@@ -2238,7 +2238,7 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>7.463150549536905e-08</v>
+        <v>7.463150549536845e-08</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
@@ -2299,7 +2299,7 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>6.301819192898289e-06</v>
+        <v>6.301819192898404e-06</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
@@ -2320,7 +2320,7 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>4.86346396611867e-06</v>
+        <v>4.863463966118776e-06</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
@@ -2341,7 +2341,7 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>1.533143450546697e-05</v>
+        <v>1.53314345054673e-05</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
@@ -2362,7 +2362,7 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>1.533143450546697e-05</v>
+        <v>1.53314345054673e-05</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -2404,7 +2404,7 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>4.393060360723199e-08</v>
+        <v>4.393060360723202e-08</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
@@ -2425,7 +2425,7 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>1.346512471990188e-05</v>
+        <v>1.346512471990197e-05</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
@@ -2780,7 +2780,7 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>1.533143450546697e-05</v>
+        <v>1.53314345054673e-05</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
@@ -2801,7 +2801,7 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>5.142264331574077e-08</v>
+        <v>5.142264331575086e-08</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>1.533143450546697e-05</v>
+        <v>1.53314345054673e-05</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
@@ -3133,7 +3133,7 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>2.048077302484792e-05</v>
+        <v>2.04807730248483e-05</v>
       </c>
       <c r="D131" t="inlineStr">
         <is>
@@ -3154,7 +3154,7 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>4.435081218854813e-06</v>
+        <v>4.435081218854969e-06</v>
       </c>
       <c r="D132" t="inlineStr">
         <is>
@@ -3466,7 +3466,7 @@
         </is>
       </c>
       <c r="C148" t="n">
-        <v>4.86346396611867e-06</v>
+        <v>4.863463966118776e-06</v>
       </c>
       <c r="D148" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
         </is>
       </c>
       <c r="C152" t="n">
-        <v>2.816695234511999e-07</v>
+        <v>2.816695234512e-07</v>
       </c>
       <c r="D152" t="inlineStr">
         <is>
@@ -3588,7 +3588,7 @@
         </is>
       </c>
       <c r="C154" t="n">
-        <v>5.146112383188477e-06</v>
+        <v>5.146112383188479e-06</v>
       </c>
       <c r="D154" t="inlineStr">
         <is>
@@ -3651,7 +3651,7 @@
         </is>
       </c>
       <c r="C157" t="n">
-        <v>8.997513026970909e-07</v>
+        <v>8.997513026971002e-07</v>
       </c>
       <c r="D157" t="inlineStr">
         <is>
@@ -3693,7 +3693,7 @@
         </is>
       </c>
       <c r="C159" t="n">
-        <v>3.07742668110825e-06</v>
+        <v>3.077426681108088e-06</v>
       </c>
       <c r="D159" t="inlineStr">
         <is>
@@ -3756,7 +3756,7 @@
         </is>
       </c>
       <c r="C162" t="n">
-        <v>4.433733428107307e-06</v>
+        <v>4.433733428107461e-06</v>
       </c>
       <c r="D162" t="inlineStr">
         <is>
@@ -3777,7 +3777,7 @@
         </is>
       </c>
       <c r="C163" t="n">
-        <v>5.2516919922559e-06</v>
+        <v>5.251691992255855e-06</v>
       </c>
       <c r="D163" t="inlineStr">
         <is>
@@ -3880,7 +3880,7 @@
         </is>
       </c>
       <c r="C168" t="n">
-        <v>1.169790846624e-06</v>
+        <v>1.169790846624001e-06</v>
       </c>
       <c r="D168" t="inlineStr">
         <is>
@@ -3941,7 +3941,7 @@
         </is>
       </c>
       <c r="C171" t="n">
-        <v>3.368663459759999e-07</v>
+        <v>3.36866345976e-07</v>
       </c>
       <c r="D171" t="inlineStr">
         <is>
@@ -4149,7 +4149,7 @@
         </is>
       </c>
       <c r="C181" t="n">
-        <v>4.894491097709419e-05</v>
+        <v>4.894491097709381e-05</v>
       </c>
       <c r="D181" t="inlineStr">
         <is>
@@ -4336,7 +4336,7 @@
         </is>
       </c>
       <c r="C190" t="n">
-        <v>2.674526857487998e-08</v>
+        <v>2.674526857488003e-08</v>
       </c>
       <c r="D190" t="inlineStr">
         <is>
@@ -4399,7 +4399,7 @@
         </is>
       </c>
       <c r="C193" t="n">
-        <v>1.567124798980799e-08</v>
+        <v>1.5671247989808e-08</v>
       </c>
       <c r="D193" t="inlineStr">
         <is>
@@ -4441,7 +4441,7 @@
         </is>
       </c>
       <c r="C195" t="n">
-        <v>4.433733428107307e-06</v>
+        <v>4.433733428107461e-06</v>
       </c>
       <c r="D195" t="inlineStr">
         <is>
@@ -4462,7 +4462,7 @@
         </is>
       </c>
       <c r="C196" t="n">
-        <v>4.433733428107307e-06</v>
+        <v>4.433733428107461e-06</v>
       </c>
       <c r="D196" t="inlineStr">
         <is>
@@ -4502,7 +4502,7 @@
         </is>
       </c>
       <c r="C198" t="n">
-        <v>8.777148687000001e-08</v>
+        <v>8.777148686999997e-08</v>
       </c>
       <c r="D198" t="inlineStr">
         <is>
@@ -4628,7 +4628,7 @@
         </is>
       </c>
       <c r="C204" t="n">
-        <v>1.081489044663215e-05</v>
+        <v>1.081489044663207e-05</v>
       </c>
       <c r="D204" t="inlineStr">
         <is>
@@ -4670,7 +4670,7 @@
         </is>
       </c>
       <c r="C206" t="n">
-        <v>1.567124798980799e-06</v>
+        <v>1.5671247989808e-06</v>
       </c>
       <c r="D206" t="inlineStr">
         <is>
@@ -4691,7 +4691,7 @@
         </is>
       </c>
       <c r="C207" t="n">
-        <v>8.018692615299729e-07</v>
+        <v>8.018692615300294e-07</v>
       </c>
       <c r="D207" t="inlineStr">
         <is>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C212" t="n">
-        <v>2.4074594973e-06</v>
+        <v>2.407459497299999e-06</v>
       </c>
       <c r="D212" t="inlineStr">
         <is>
@@ -4943,7 +4943,7 @@
         </is>
       </c>
       <c r="C219" t="n">
-        <v>2.130842931728973e-06</v>
+        <v>2.130842931729123e-06</v>
       </c>
       <c r="D219" t="inlineStr">
         <is>
@@ -5065,7 +5065,7 @@
         </is>
       </c>
       <c r="C225" t="n">
-        <v>5.094411847991999e-06</v>
+        <v>5.094411847992003e-06</v>
       </c>
       <c r="D225" t="inlineStr">
         <is>
@@ -5170,7 +5170,7 @@
         </is>
       </c>
       <c r="C230" t="n">
-        <v>2.828403453658091e-07</v>
+        <v>2.828403453658057e-07</v>
       </c>
       <c r="D230" t="inlineStr">
         <is>
@@ -5191,7 +5191,7 @@
         </is>
       </c>
       <c r="C231" t="n">
-        <v>2.048077302484792e-05</v>
+        <v>2.04807730248483e-05</v>
       </c>
       <c r="D231" t="inlineStr">
         <is>
@@ -5233,7 +5233,7 @@
         </is>
       </c>
       <c r="C233" t="n">
-        <v>2.354566314384545e-08</v>
+        <v>2.354566314386172e-08</v>
       </c>
       <c r="D233" t="inlineStr">
         <is>
@@ -5456,7 +5456,7 @@
         </is>
       </c>
       <c r="C244" t="n">
-        <v>1.436752891940833e-08</v>
+        <v>1.436752891940836e-08</v>
       </c>
       <c r="D244" t="inlineStr">
         <is>
@@ -5559,7 +5559,7 @@
         </is>
       </c>
       <c r="C249" t="n">
-        <v>1.533143450546697e-05</v>
+        <v>1.53314345054673e-05</v>
       </c>
       <c r="D249" t="inlineStr">
         <is>
@@ -5683,7 +5683,7 @@
         </is>
       </c>
       <c r="C255" t="n">
-        <v>2.4074594973e-06</v>
+        <v>2.407459497299999e-06</v>
       </c>
       <c r="D255" t="inlineStr">
         <is>
@@ -5746,7 +5746,7 @@
         </is>
       </c>
       <c r="C258" t="n">
-        <v>4.945144969682013e-06</v>
+        <v>4.945144969682073e-06</v>
       </c>
       <c r="D258" t="inlineStr">
         <is>
@@ -5807,7 +5807,7 @@
         </is>
       </c>
       <c r="C261" t="n">
-        <v>3.234118665314228e-07</v>
+        <v>3.234118665314224e-07</v>
       </c>
       <c r="D261" t="inlineStr">
         <is>
@@ -6463,7 +6463,7 @@
         </is>
       </c>
       <c r="C293" t="n">
-        <v>1.461325492681854e-07</v>
+        <v>1.461325492681836e-07</v>
       </c>
       <c r="D293" t="inlineStr">
         <is>
@@ -6585,7 +6585,7 @@
         </is>
       </c>
       <c r="C299" t="n">
-        <v>4.265124784991903e-06</v>
+        <v>4.265124784991902e-06</v>
       </c>
       <c r="D299" t="inlineStr">
         <is>
@@ -6606,7 +6606,7 @@
         </is>
       </c>
       <c r="C300" t="n">
-        <v>2.166232669495852e-07</v>
+        <v>2.166232669503957e-07</v>
       </c>
       <c r="D300" t="inlineStr">
         <is>
@@ -6648,7 +6648,7 @@
         </is>
       </c>
       <c r="C302" t="n">
-        <v>1.486343890656e-06</v>
+        <v>1.486343890656001e-06</v>
       </c>
       <c r="D302" t="inlineStr">
         <is>
@@ -6877,7 +6877,7 @@
         </is>
       </c>
       <c r="C313" t="n">
-        <v>2.95479864234e-07</v>
+        <v>2.954798642339999e-07</v>
       </c>
       <c r="D313" t="inlineStr">
         <is>
@@ -7022,7 +7022,7 @@
         </is>
       </c>
       <c r="C320" t="n">
-        <v>2.048077302484792e-05</v>
+        <v>2.04807730248483e-05</v>
       </c>
       <c r="D320" t="inlineStr">
         <is>
@@ -7085,7 +7085,7 @@
         </is>
       </c>
       <c r="C323" t="n">
-        <v>2.831656841951999e-06</v>
+        <v>2.831656841952e-06</v>
       </c>
       <c r="D323" t="inlineStr">
         <is>
@@ -7253,7 +7253,7 @@
         </is>
       </c>
       <c r="C331" t="n">
-        <v>7.660250070600001e-07</v>
+        <v>7.660250070599997e-07</v>
       </c>
       <c r="D331" t="inlineStr">
         <is>
@@ -7358,7 +7358,7 @@
         </is>
       </c>
       <c r="C336" t="n">
-        <v>2.066737431555275e-06</v>
+        <v>2.066737431555269e-06</v>
       </c>
       <c r="D336" t="inlineStr">
         <is>
@@ -7440,7 +7440,7 @@
         </is>
       </c>
       <c r="C340" t="n">
-        <v>1.044570341792724e-06</v>
+        <v>1.044570341792799e-06</v>
       </c>
       <c r="D340" t="inlineStr">
         <is>
@@ -7854,7 +7854,7 @@
         </is>
       </c>
       <c r="C360" t="n">
-        <v>4.433733428107307e-06</v>
+        <v>4.433733428107461e-06</v>
       </c>
       <c r="D360" t="inlineStr">
         <is>
@@ -8371,7 +8371,7 @@
         </is>
       </c>
       <c r="C385" t="n">
-        <v>4.86346396611867e-06</v>
+        <v>4.863463966118776e-06</v>
       </c>
       <c r="D385" t="inlineStr">
         <is>
@@ -8497,7 +8497,7 @@
         </is>
       </c>
       <c r="C391" t="n">
-        <v>5.738456305779496e-05</v>
+        <v>5.738456305779478e-05</v>
       </c>
       <c r="D391" t="inlineStr">
         <is>
@@ -8663,7 +8663,7 @@
         </is>
       </c>
       <c r="C399" t="n">
-        <v>3.667332433669257e-05</v>
+        <v>3.667332433669033e-05</v>
       </c>
       <c r="D399" t="inlineStr">
         <is>
@@ -9378,7 +9378,7 @@
         </is>
       </c>
       <c r="C434" t="n">
-        <v>8.15701307575038e-05</v>
+        <v>8.157013075750382e-05</v>
       </c>
       <c r="D434" t="inlineStr">
         <is>
@@ -9546,7 +9546,7 @@
         </is>
       </c>
       <c r="C442" t="n">
-        <v>3.691040058493541e-06</v>
+        <v>3.691040058493523e-06</v>
       </c>
       <c r="D442" t="inlineStr">
         <is>
@@ -9567,7 +9567,7 @@
         </is>
       </c>
       <c r="C443" t="n">
-        <v>1.330651065564092e-07</v>
+        <v>1.330651065567433e-07</v>
       </c>
       <c r="D443" t="inlineStr">
         <is>
@@ -9672,7 +9672,7 @@
         </is>
       </c>
       <c r="C448" t="n">
-        <v>1.533143450546697e-05</v>
+        <v>1.53314345054673e-05</v>
       </c>
       <c r="D448" t="inlineStr">
         <is>
@@ -9714,7 +9714,7 @@
         </is>
       </c>
       <c r="C450" t="n">
-        <v>4.898477223680456e-06</v>
+        <v>4.898477223680425e-06</v>
       </c>
       <c r="D450" t="inlineStr">
         <is>
@@ -9882,7 +9882,7 @@
         </is>
       </c>
       <c r="C458" t="n">
-        <v>2.048077302484792e-05</v>
+        <v>2.04807730248483e-05</v>
       </c>
       <c r="D458" t="inlineStr">
         <is>
@@ -10256,7 +10256,7 @@
         </is>
       </c>
       <c r="C476" t="n">
-        <v>7.360403696506622e-07</v>
+        <v>7.360403696506623e-07</v>
       </c>
       <c r="D476" t="inlineStr">
         <is>
@@ -10502,7 +10502,7 @@
         </is>
       </c>
       <c r="C488" t="n">
-        <v>5.738456305779496e-05</v>
+        <v>5.738456305779478e-05</v>
       </c>
       <c r="D488" t="inlineStr">
         <is>
@@ -10565,7 +10565,7 @@
         </is>
       </c>
       <c r="C491" t="n">
-        <v>3.640646677007991e-07</v>
+        <v>3.640646677008013e-07</v>
       </c>
       <c r="D491" t="inlineStr">
         <is>
@@ -10897,7 +10897,7 @@
         </is>
       </c>
       <c r="C507" t="n">
-        <v>1.56417798853505e-05</v>
+        <v>1.564177988535066e-05</v>
       </c>
       <c r="D507" t="inlineStr">
         <is>
@@ -11164,7 +11164,7 @@
         </is>
       </c>
       <c r="C520" t="n">
-        <v>5.860564011794284e-08</v>
+        <v>5.860564011795175e-08</v>
       </c>
       <c r="D520" t="inlineStr">
         <is>
@@ -11185,7 +11185,7 @@
         </is>
       </c>
       <c r="C521" t="n">
-        <v>5.693621816142285e-05</v>
+        <v>5.693621816142344e-05</v>
       </c>
       <c r="D521" t="inlineStr">
         <is>
@@ -11288,7 +11288,7 @@
         </is>
       </c>
       <c r="C526" t="n">
-        <v>2.232607540392707e-06</v>
+        <v>2.232607540392681e-06</v>
       </c>
       <c r="D526" t="inlineStr">
         <is>
@@ -11750,7 +11750,7 @@
         </is>
       </c>
       <c r="C548" t="n">
-        <v>5.401275601200001e-08</v>
+        <v>5.401275601199998e-08</v>
       </c>
       <c r="D548" t="inlineStr">
         <is>
@@ -11830,7 +11830,7 @@
         </is>
       </c>
       <c r="C552" t="n">
-        <v>1.28000501950529e-09</v>
+        <v>1.280005019508501e-09</v>
       </c>
       <c r="D552" t="inlineStr">
         <is>
@@ -12538,7 +12538,7 @@
         </is>
       </c>
       <c r="C586" t="n">
-        <v>2.936167069832115e-07</v>
+        <v>2.936167069831935e-07</v>
       </c>
       <c r="D586" t="inlineStr">
         <is>
@@ -13017,7 +13017,7 @@
         </is>
       </c>
       <c r="C609" t="n">
-        <v>6.694282706385579e-07</v>
+        <v>6.694282706385589e-07</v>
       </c>
       <c r="D609" t="inlineStr">
         <is>
@@ -13139,7 +13139,7 @@
         </is>
       </c>
       <c r="C615" t="n">
-        <v>1.135735642262811e-07</v>
+        <v>1.135735642262741e-07</v>
       </c>
       <c r="D615" t="inlineStr">
         <is>
@@ -13259,7 +13259,7 @@
         </is>
       </c>
       <c r="C621" t="n">
-        <v>2.182702790533646e-08</v>
+        <v>2.182702790541812e-08</v>
       </c>
       <c r="D621" t="inlineStr">
         <is>
@@ -13507,7 +13507,7 @@
         </is>
       </c>
       <c r="C633" t="n">
-        <v>3.006296338317791e-06</v>
+        <v>3.006296338317827e-06</v>
       </c>
       <c r="D633" t="inlineStr">
         <is>
@@ -13839,7 +13839,7 @@
         </is>
       </c>
       <c r="C649" t="n">
-        <v>5.92442404323996e-07</v>
+        <v>5.924424043239959e-07</v>
       </c>
       <c r="D649" t="inlineStr">
         <is>
@@ -13923,7 +13923,7 @@
         </is>
       </c>
       <c r="C653" t="n">
-        <v>5.401275601200001e-08</v>
+        <v>5.401275601199998e-08</v>
       </c>
       <c r="D653" t="inlineStr">
         <is>
@@ -14085,7 +14085,7 @@
         </is>
       </c>
       <c r="C661" t="n">
-        <v>1.28000501950529e-09</v>
+        <v>1.280005019508501e-09</v>
       </c>
       <c r="D661" t="inlineStr">
         <is>
@@ -14375,7 +14375,7 @@
         </is>
       </c>
       <c r="C675" t="n">
-        <v>1.28000501950529e-09</v>
+        <v>1.280005019508501e-09</v>
       </c>
       <c r="D675" t="inlineStr">
         <is>
@@ -14951,7 +14951,7 @@
         </is>
       </c>
       <c r="C703" t="n">
-        <v>8.751351992114283e-08</v>
+        <v>8.751351992115177e-08</v>
       </c>
       <c r="D703" t="inlineStr">
         <is>
@@ -15014,7 +15014,7 @@
         </is>
       </c>
       <c r="C706" t="n">
-        <v>1.410190451687396e-07</v>
+        <v>1.410190451687395e-07</v>
       </c>
       <c r="D706" t="inlineStr">
         <is>
@@ -16217,7 +16217,7 @@
         </is>
       </c>
       <c r="C765" t="n">
-        <v>0.0002048077302484792</v>
+        <v>0.000204807730248483</v>
       </c>
       <c r="D765" t="inlineStr">
         <is>
@@ -16255,7 +16255,7 @@
         </is>
       </c>
       <c r="C767" t="n">
-        <v>2.803416671328357e-06</v>
+        <v>2.803416671328333e-06</v>
       </c>
       <c r="D767" t="inlineStr">
         <is>
@@ -16297,7 +16297,7 @@
         </is>
       </c>
       <c r="C769" t="n">
-        <v>2.048077302484792e-05</v>
+        <v>2.04807730248483e-05</v>
       </c>
       <c r="D769" t="inlineStr">
         <is>
@@ -16318,7 +16318,7 @@
         </is>
       </c>
       <c r="C770" t="n">
-        <v>2.048077302484792e-05</v>
+        <v>2.04807730248483e-05</v>
       </c>
       <c r="D770" t="inlineStr">
         <is>
@@ -16339,7 +16339,7 @@
         </is>
       </c>
       <c r="C771" t="n">
-        <v>2.048077302484792e-05</v>
+        <v>2.04807730248483e-05</v>
       </c>
       <c r="D771" t="inlineStr">
         <is>
@@ -16484,7 +16484,7 @@
         </is>
       </c>
       <c r="C778" t="n">
-        <v>4.86346396611867e-06</v>
+        <v>4.863463966118776e-06</v>
       </c>
       <c r="D778" t="inlineStr">
         <is>
@@ -17298,7 +17298,7 @@
         </is>
       </c>
       <c r="C818" t="n">
-        <v>2.913186550296131e-06</v>
+        <v>2.913186550296113e-06</v>
       </c>
       <c r="D818" t="inlineStr">
         <is>
@@ -17794,7 +17794,7 @@
         </is>
       </c>
       <c r="C842" t="n">
-        <v>3.564328880112524e-06</v>
+        <v>3.564328880112488e-06</v>
       </c>
       <c r="D842" t="inlineStr">
         <is>
@@ -18042,7 +18042,7 @@
         </is>
       </c>
       <c r="C854" t="n">
-        <v>2.048077302484792e-05</v>
+        <v>2.04807730248483e-05</v>
       </c>
       <c r="D854" t="inlineStr">
         <is>
@@ -18410,7 +18410,7 @@
         </is>
       </c>
       <c r="C872" t="n">
-        <v>2.328308822606448e-06</v>
+        <v>2.328308822606446e-06</v>
       </c>
       <c r="D872" t="inlineStr">
         <is>
@@ -19193,7 +19193,7 @@
         </is>
       </c>
       <c r="C911" t="n">
-        <v>9.337869477336262e-06</v>
+        <v>9.337869477336206e-06</v>
       </c>
       <c r="D911" t="inlineStr">
         <is>
@@ -19403,7 +19403,7 @@
         </is>
       </c>
       <c r="C921" t="n">
-        <v>2.048077302484792e-05</v>
+        <v>2.04807730248483e-05</v>
       </c>
       <c r="D921" t="inlineStr">
         <is>
@@ -19487,7 +19487,7 @@
         </is>
       </c>
       <c r="C925" t="n">
-        <v>2.374072297652929e-05</v>
+        <v>2.374072297652944e-05</v>
       </c>
       <c r="D925" t="inlineStr">
         <is>
@@ -19586,7 +19586,7 @@
         </is>
       </c>
       <c r="C930" t="n">
-        <v>2.048077302484792e-05</v>
+        <v>2.04807730248483e-05</v>
       </c>
       <c r="D930" t="inlineStr">
         <is>
@@ -19752,7 +19752,7 @@
         </is>
       </c>
       <c r="C938" t="n">
-        <v>2.048077302484792e-05</v>
+        <v>2.04807730248483e-05</v>
       </c>
       <c r="D938" t="inlineStr">
         <is>

</xml_diff>